<commit_message>
Add ghoul poses; ghoul takes one slot, wolf takes two
- Three user-provided ghoul images become poses: slash (lunging claw),
  slash_2 (crouched roar, picked at random as an alternate attack) and
  hit (head thrown back), scaled from the hit pose height.
- Monster footprint swapped: ghoul 2 -> 1 slot (front), wolf 1 -> 2
  (middle + back). Only the two 차지칸 cells in balance.xlsx were
  changed in place; stage_01, the test roster, codex subtitles and the
  placement tests follow the new layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aytw3hj7boqn3SZ5GP5ti
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
         <v>240</v>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
         <v>400</v>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>구울(전방·중앙) + 늑대(후방). 배치는 스테이지 에디터</t>
+          <t>구울(전방) + 늑대(중앙·후방). 배치는 스테이지 에디터</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add human enemy AU army soldier (army_m)
- New character from the user's 9-image package: base image rigged into
  a 32-frame idle; poses for pistol/SMG fire (shot, shot_pistol,
  shot_smg), slash, cast (point_up), hit, miss, tired (16-frame
  breathing rig) and dead, all at the base image scale.
- Added to the enemy list: one appended row in balance.xlsx 몬스터
  (role 인간, ranged, pistol/smg/knife, placeholder stats), a skill kit
  in monster_skills.json and a codex entry.
- Death rule: enemies whose role is 인간 fall with their dead pose;
  only monsters burn away. Stage placement left to the stage editor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aytw3hj7boqn3SZ5GP5ti
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -1067,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1396,6 +1396,78 @@
       </c>
       <c r="R4" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>army_m</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AU군 병사</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>인간</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>원거리</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>pistol, smg, knife</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>178</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>army_m</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>오른쪽</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>5</v>
+      </c>
+      <c r="R5" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add human enemy AU army bigman; lay dead bodies on their shadows
- bigman from the user's 9-image package: base rigged into a 32-frame
  idle, tired with a breathing loop, and the same pose set as army_m.
  The images were drawn at different scales, so each pose is scaled by
  the average of its uniform-area and boots/gloves-area ratio to idle.
- Registered as a human enemy (dead pose on death): one appended row in
  balance.xlsx 몬스터 (melee brute, placeholder stats), skill kit and
  codex entry.
- Lying dead poses put the foot line 30% of the body thickness above the
  lowest pixel, so bodies rest on the round shadow instead of floating.
  Applied to all eight dead poses; the poses tool now does the same.
- Debug: --autoplay=burn[:sec[:all]] also kills allies with "all".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aytw3hj7boqn3SZ5GP5ti
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -1067,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1468,6 +1468,78 @@
       </c>
       <c r="R5" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bigman</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AU군 거한</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>인간</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>근접</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>120</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>combat_knife, smg, pistol</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>205</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>bigman</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>오른쪽</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>aggressive</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>